<commit_message>
Add target list: OT
</commit_message>
<xml_diff>
--- a/data/reports/ot.xlsx
+++ b/data/reports/ot.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -624,11 +624,7 @@
           <t>541512</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Computer Systems Design Services</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Primary</t>
@@ -642,11 +638,7 @@
           <t>541611</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Administrative Management and General Management Consulting Services</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Primary</t>
@@ -660,17 +652,69 @@
           <t>541618</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Other Management Consulting Services</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>541690</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>541330</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>541519</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>541513</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -746,7 +790,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>OT Cybersecurity</t>
+          <t>OT, Cybersecurity, Consulting, Advisory</t>
         </is>
       </c>
     </row>
@@ -758,7 +802,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
@@ -770,7 +814,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09T12:25:03.255819+00:00</t>
+          <t>2026-07-09T13:09:24.222013+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>